<commit_message>
Přidán nový díl Magnet proporciální chlazení (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,22 +439,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>844</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Proporciální ventil chlazení</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1517815</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Proporciální ventil chlazení</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1517815</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Magnet proporciální chlazení</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1994523</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Elektrické ovládání pro chlazení (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,22 +453,36 @@
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>844</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Magnet proporciální chlazení</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1994523</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Magnet proporciální chlazení</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1994523</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Elektrické ovládání pro chlazení</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1767947</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Kabel ovládání válce řazení (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,22 +467,40 @@
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>844</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Elektrické ovládání pro chlazení</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1767947</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Elektrické ovládání pro chlazení</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1767947</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kabel ovládání válce řazení</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2192995</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>do vzduchové kostky kabel</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Zásuvka nabíjecí 24V USB (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,22 +481,40 @@
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>844</t>
-        </is>
+      <c r="A5" t="n">
+        <v>844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>Kabel ovládání válce řazení</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2192995</t>
-        </is>
+      <c r="C5" t="n">
+        <v>2192995</v>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>do vzduchové kostky kabel</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>814</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Zásuvka nabíjecí 24V USB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1867116</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>do vzduchové kostky kabel</t>
         </is>

</xml_diff>

<commit_message>
Přidán nový díl Čidlo hladiny oleje (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,26 +499,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>814</t>
-        </is>
+      <c r="A6" t="n">
+        <v>814</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>Zásuvka nabíjecí 24V USB</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1867116</t>
-        </is>
+      <c r="C6" t="n">
+        <v>1867116</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>do vzduchové kostky kabel</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Čidlo hladiny oleje</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1531719</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Čidlo překročení teploty ložiska  (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,22 +517,36 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>844</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Čidlo hladiny oleje</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1531719</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Čidlo hladiny oleje</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1531719</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Čidlo překročení teploty ložiska</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1683202</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Naftoznak displej C6 LS AKSEL (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,22 +531,36 @@
       <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>844</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Čidlo překročení teploty ložiska</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1683202</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Čidlo překročení teploty ložiska</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1683202</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Naftoznak displej C6 LS AKSEL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1864416</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Řídící jednotka scr modulu (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,22 +545,40 @@
       <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>844</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Naftoznak displej C6 LS AKSEL</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1864416</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Naftoznak displej C6 LS AKSEL</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1864416</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Řídící jednotka scr modulu</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1517016</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rámový blok</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Kabel převodovky s konektory (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,26 +559,40 @@
       <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>844</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Řídící jednotka scr modulu</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1517016</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rámový blok</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Řídící jednotka scr modulu</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1517016</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Rámový blok</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kabel převodovky s konektory</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1766981</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Kabeláž elektrická motoru MTU (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,22 +577,36 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>844</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kabel převodovky s konektory</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1766981</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Kabel převodovky s konektory</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1766981</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kabeláž elektrická motoru MTU</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1531754</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Kabeláž motoru  (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,22 +591,40 @@
       <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>844</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kabeláž elektrická motoru MTU</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1531754</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Kabeláž elektrická motoru MTU</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1531754</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kabeláž motoru</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1767958</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Na motoru kabeláž</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Kompresor klimatizace  (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,26 +605,40 @@
       <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>844</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kabeláž motoru</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1767958</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Na motoru kabeláž</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Kabeláž motoru</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1767958</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Na motoru kabeláž</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kompresor klimatizace</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1646752</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Capos kondenzátory  (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,22 +623,36 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="n">
+        <v>844</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kompresor klimatizace</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1646752</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Kompresor klimatizace</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1646752</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Capos kondenzátory</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2077086</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidán nový díl Měnič DC/DC capos  (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,22 +637,40 @@
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="n">
+        <v>844</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Capos kondenzátory</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2077086</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>844</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Capos kondenzátory</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2077086</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Měnič DC/DC capos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2018024</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Capos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Úprava/Smazání dílů v tabulce (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -648,23 +648,23 @@
       <c r="C15" t="n">
         <v>2077086</v>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Capos</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>844</t>
-        </is>
+      <c r="A16" t="n">
+        <v>844</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>Měnič DC/DC capos</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2018024</t>
-        </is>
+      <c r="C16" t="n">
+        <v>2018024</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Přidán nový díl Regulátor stěračů BER-2 (autor: Radek)
</commit_message>
<xml_diff>
--- a/SEZNAM_DILU.xlsx
+++ b/SEZNAM_DILU.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -668,6 +668,28 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Regulátor stěračů BER-2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1660961</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Posteor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>